<commit_message>
Update dataset: replace task-sici with task-rest, add EMG data
</commit_message>
<xml_diff>
--- a/nibs-das_examples/mep_example/collated_participant_data/nibs-das_mep_exampledata_2026-02-04.xlsx
+++ b/nibs-das_examples/mep_example/collated_participant_data/nibs-das_mep_exampledata_2026-02-04.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://deakin365-my.sharepoint.com/personal/michael_barham_deakin_edu_au/Documents/Desktop/Research/Big NIBS Data/Projects/2026_NIBS-DAS/NIBS-DAS_examples/2026-02-01/NIBS-DAS_mep_example/collated_participant_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielcorp/Dropbox/2016_BigTMSdata/0_Projects/0_2023_NIBS-DAS/NewFolderStructure_Oct25/GitClone/nibs-das_repo/nibs-das_examples/mep_example/collated_participant_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{4D659B1F-5006-3947-A93D-82DE7168EF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEEF7209-DB1E-4926-AC7C-720E71375BC9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3C40D9-6B3C-E946-90A9-3507065654A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1760" yWindow="1000" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -627,28 +627,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{185C0B89-D493-404E-B623-16DE972B9450}">
   <dimension ref="A1:T401"/>
-  <sheetFormatPr defaultColWidth="9.3046875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.69140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="6.3046875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.84375" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.3046875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.15234375" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.3046875" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.3046875" style="10"/>
-    <col min="10" max="10" width="12.15234375" style="8" customWidth="1"/>
-    <col min="11" max="11" width="12.53515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.53515625" style="8" customWidth="1"/>
-    <col min="13" max="13" width="11.3828125" style="8" customWidth="1"/>
-    <col min="14" max="14" width="12.15234375" style="8" customWidth="1"/>
-    <col min="15" max="15" width="9.69140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="6.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.28515625" style="10"/>
+    <col min="10" max="10" width="12.140625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" style="8" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" style="8" customWidth="1"/>
+    <col min="14" max="14" width="12.140625" style="8" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="11.53515625" style="9" customWidth="1"/>
-    <col min="19" max="20" width="13.69140625" style="9" customWidth="1"/>
-    <col min="21" max="16384" width="9.3046875" style="8"/>
+    <col min="17" max="18" width="11.5703125" style="9" customWidth="1"/>
+    <col min="19" max="20" width="13.7109375" style="9" customWidth="1"/>
+    <col min="21" max="16384" width="9.28515625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -710,7 +710,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -772,7 +772,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -834,7 +834,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -896,7 +896,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -958,7 +958,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="19" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>11</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>11</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>11</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>11</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>11</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="33" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>11</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>11</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>11</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>11</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>11</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>11</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>11</v>
       </c>
@@ -3128,7 +3128,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:20" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>11</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>12</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>12</v>
       </c>
@@ -3314,7 +3314,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>12</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>12</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>12</v>
       </c>
@@ -3562,7 +3562,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="48" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>12</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>12</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
@@ -3748,7 +3748,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="51" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>12</v>
       </c>
@@ -3810,7 +3810,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>12</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>12</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -4182,7 +4182,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>12</v>
       </c>
@@ -4244,7 +4244,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>12</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>12</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="61" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>12</v>
       </c>
@@ -4430,7 +4430,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>12</v>
       </c>
@@ -4492,7 +4492,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>12</v>
       </c>
@@ -4554,7 +4554,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>12</v>
       </c>
@@ -4616,7 +4616,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>12</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>12</v>
       </c>
@@ -4740,7 +4740,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>12</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>12</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>12</v>
       </c>
@@ -4926,7 +4926,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>12</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>12</v>
       </c>
@@ -5050,7 +5050,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>12</v>
       </c>
@@ -5112,7 +5112,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>12</v>
       </c>
@@ -5174,7 +5174,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>12</v>
       </c>
@@ -5236,7 +5236,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>12</v>
       </c>
@@ -5298,7 +5298,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>12</v>
       </c>
@@ -5360,7 +5360,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>12</v>
       </c>
@@ -5422,7 +5422,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>12</v>
       </c>
@@ -5484,7 +5484,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>12</v>
       </c>
@@ -5546,7 +5546,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="80" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>12</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="81" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>12</v>
       </c>
@@ -5670,7 +5670,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>13</v>
       </c>
@@ -5732,7 +5732,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>13</v>
       </c>
@@ -5794,7 +5794,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>13</v>
       </c>
@@ -5856,7 +5856,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>13</v>
       </c>
@@ -5918,7 +5918,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>13</v>
       </c>
@@ -5980,7 +5980,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>13</v>
       </c>
@@ -6042,7 +6042,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>13</v>
       </c>
@@ -6104,7 +6104,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>13</v>
       </c>
@@ -6166,7 +6166,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>13</v>
       </c>
@@ -6228,7 +6228,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>13</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>13</v>
       </c>
@@ -6352,7 +6352,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>13</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>13</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>13</v>
       </c>
@@ -6538,7 +6538,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>13</v>
       </c>
@@ -6600,7 +6600,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>13</v>
       </c>
@@ -6662,7 +6662,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>13</v>
       </c>
@@ -6724,7 +6724,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="99" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>13</v>
       </c>
@@ -6786,7 +6786,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>13</v>
       </c>
@@ -6848,7 +6848,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>13</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>13</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>13</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>13</v>
       </c>
@@ -7096,7 +7096,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>13</v>
       </c>
@@ -7158,7 +7158,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>13</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>13</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>13</v>
       </c>
@@ -7344,7 +7344,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>13</v>
       </c>
@@ -7406,7 +7406,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>13</v>
       </c>
@@ -7468,7 +7468,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>13</v>
       </c>
@@ -7530,7 +7530,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>13</v>
       </c>
@@ -7592,7 +7592,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>13</v>
       </c>
@@ -7654,7 +7654,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="114" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>13</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>13</v>
       </c>
@@ -7778,7 +7778,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>13</v>
       </c>
@@ -7840,7 +7840,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>13</v>
       </c>
@@ -7902,7 +7902,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>13</v>
       </c>
@@ -7964,7 +7964,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>13</v>
       </c>
@@ -8026,7 +8026,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>13</v>
       </c>
@@ -8088,7 +8088,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>13</v>
       </c>
@@ -8150,7 +8150,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="122" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>14</v>
       </c>
@@ -8212,7 +8212,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>14</v>
       </c>
@@ -8274,7 +8274,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>14</v>
       </c>
@@ -8336,7 +8336,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>14</v>
       </c>
@@ -8398,7 +8398,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>14</v>
       </c>
@@ -8460,7 +8460,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="127" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>14</v>
       </c>
@@ -8522,7 +8522,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>14</v>
       </c>
@@ -8584,7 +8584,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>14</v>
       </c>
@@ -8646,7 +8646,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>14</v>
       </c>
@@ -8708,7 +8708,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>14</v>
       </c>
@@ -8770,7 +8770,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>14</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>14</v>
       </c>
@@ -8894,7 +8894,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>14</v>
       </c>
@@ -8956,7 +8956,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>14</v>
       </c>
@@ -9018,7 +9018,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>14</v>
       </c>
@@ -9080,7 +9080,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="137" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>14</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>14</v>
       </c>
@@ -9204,7 +9204,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>14</v>
       </c>
@@ -9266,7 +9266,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>14</v>
       </c>
@@ -9328,7 +9328,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="141" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>14</v>
       </c>
@@ -9390,7 +9390,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>14</v>
       </c>
@@ -9452,7 +9452,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>14</v>
       </c>
@@ -9514,7 +9514,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>14</v>
       </c>
@@ -9576,7 +9576,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>14</v>
       </c>
@@ -9638,7 +9638,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="146" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>14</v>
       </c>
@@ -9700,7 +9700,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>14</v>
       </c>
@@ -9762,7 +9762,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>14</v>
       </c>
@@ -9824,7 +9824,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>14</v>
       </c>
@@ -9886,7 +9886,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>14</v>
       </c>
@@ -9948,7 +9948,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>14</v>
       </c>
@@ -10010,7 +10010,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>14</v>
       </c>
@@ -10072,7 +10072,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>14</v>
       </c>
@@ -10134,7 +10134,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="154" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>14</v>
       </c>
@@ -10196,7 +10196,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>14</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>14</v>
       </c>
@@ -10320,7 +10320,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>14</v>
       </c>
@@ -10382,7 +10382,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>14</v>
       </c>
@@ -10444,7 +10444,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>14</v>
       </c>
@@ -10506,7 +10506,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>14</v>
       </c>
@@ -10568,7 +10568,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>14</v>
       </c>
@@ -10630,7 +10630,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>15</v>
       </c>
@@ -10692,7 +10692,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>15</v>
       </c>
@@ -10754,7 +10754,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>15</v>
       </c>
@@ -10816,7 +10816,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>15</v>
       </c>
@@ -10878,7 +10878,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>15</v>
       </c>
@@ -10940,7 +10940,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
         <v>15</v>
       </c>
@@ -11002,7 +11002,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
         <v>15</v>
       </c>
@@ -11064,7 +11064,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
         <v>15</v>
       </c>
@@ -11126,7 +11126,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="170" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
         <v>15</v>
       </c>
@@ -11188,7 +11188,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
         <v>15</v>
       </c>
@@ -11250,7 +11250,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>15</v>
       </c>
@@ -11312,7 +11312,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>15</v>
       </c>
@@ -11374,7 +11374,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="174" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
         <v>15</v>
       </c>
@@ -11436,7 +11436,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="175" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
         <v>15</v>
       </c>
@@ -11498,7 +11498,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
         <v>15</v>
       </c>
@@ -11560,7 +11560,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
         <v>15</v>
       </c>
@@ -11622,7 +11622,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
         <v>15</v>
       </c>
@@ -11684,7 +11684,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="179" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
         <v>15</v>
       </c>
@@ -11746,7 +11746,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="180" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
         <v>15</v>
       </c>
@@ -11808,7 +11808,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="181" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
         <v>15</v>
       </c>
@@ -11870,7 +11870,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="182" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
         <v>15</v>
       </c>
@@ -11932,7 +11932,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="183" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
         <v>15</v>
       </c>
@@ -11994,7 +11994,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="184" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
         <v>15</v>
       </c>
@@ -12056,7 +12056,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
         <v>15</v>
       </c>
@@ -12118,7 +12118,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="186" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
         <v>15</v>
       </c>
@@ -12180,7 +12180,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="187" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
         <v>15</v>
       </c>
@@ -12242,7 +12242,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
         <v>15</v>
       </c>
@@ -12304,7 +12304,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="189" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
         <v>15</v>
       </c>
@@ -12366,7 +12366,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
         <v>15</v>
       </c>
@@ -12428,7 +12428,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
         <v>15</v>
       </c>
@@ -12490,7 +12490,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="192" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
         <v>15</v>
       </c>
@@ -12552,7 +12552,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="193" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
         <v>15</v>
       </c>
@@ -12614,7 +12614,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="194" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>15</v>
       </c>
@@ -12676,7 +12676,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="195" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
         <v>15</v>
       </c>
@@ -12738,7 +12738,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
         <v>15</v>
       </c>
@@ -12800,7 +12800,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
         <v>15</v>
       </c>
@@ -12862,7 +12862,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
         <v>15</v>
       </c>
@@ -12924,7 +12924,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="199" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
         <v>15</v>
       </c>
@@ -12986,7 +12986,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="200" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="s">
         <v>15</v>
       </c>
@@ -13048,7 +13048,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="201" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
         <v>15</v>
       </c>
@@ -13110,7 +13110,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
         <v>16</v>
       </c>
@@ -13172,7 +13172,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="s">
         <v>16</v>
       </c>
@@ -13234,7 +13234,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="204" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
         <v>16</v>
       </c>
@@ -13296,7 +13296,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="205" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="s">
         <v>16</v>
       </c>
@@ -13358,7 +13358,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="206" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A206" s="1" t="s">
         <v>16</v>
       </c>
@@ -13420,7 +13420,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="207" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
         <v>16</v>
       </c>
@@ -13482,7 +13482,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="s">
         <v>16</v>
       </c>
@@ -13544,7 +13544,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="209" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
         <v>16</v>
       </c>
@@ -13606,7 +13606,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="210" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
         <v>16</v>
       </c>
@@ -13668,7 +13668,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="211" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
         <v>16</v>
       </c>
@@ -13730,7 +13730,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
         <v>16</v>
       </c>
@@ -13792,7 +13792,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="213" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
         <v>16</v>
       </c>
@@ -13854,7 +13854,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="214" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
         <v>16</v>
       </c>
@@ -13916,7 +13916,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="s">
         <v>16</v>
       </c>
@@ -13978,7 +13978,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="216" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
         <v>16</v>
       </c>
@@ -14040,7 +14040,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="217" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
         <v>16</v>
       </c>
@@ -14102,7 +14102,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
         <v>16</v>
       </c>
@@ -14164,7 +14164,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
         <v>16</v>
       </c>
@@ -14226,7 +14226,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
         <v>16</v>
       </c>
@@ -14288,7 +14288,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="221" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
         <v>16</v>
       </c>
@@ -14350,7 +14350,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="222" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
         <v>16</v>
       </c>
@@ -14412,7 +14412,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="223" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
         <v>16</v>
       </c>
@@ -14474,7 +14474,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
         <v>16</v>
       </c>
@@ -14536,7 +14536,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="225" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
         <v>16</v>
       </c>
@@ -14598,7 +14598,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
         <v>16</v>
       </c>
@@ -14660,7 +14660,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
         <v>16</v>
       </c>
@@ -14722,7 +14722,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
         <v>16</v>
       </c>
@@ -14784,7 +14784,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="229" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
         <v>16</v>
       </c>
@@ -14846,7 +14846,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
         <v>16</v>
       </c>
@@ -14908,7 +14908,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
         <v>16</v>
       </c>
@@ -14970,7 +14970,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
         <v>16</v>
       </c>
@@ -15032,7 +15032,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="233" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
         <v>16</v>
       </c>
@@ -15094,7 +15094,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="s">
         <v>16</v>
       </c>
@@ -15156,7 +15156,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="235" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
         <v>16</v>
       </c>
@@ -15218,7 +15218,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="236" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
         <v>16</v>
       </c>
@@ -15280,7 +15280,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
         <v>16</v>
       </c>
@@ -15342,7 +15342,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
         <v>16</v>
       </c>
@@ -15404,7 +15404,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="239" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
         <v>16</v>
       </c>
@@ -15466,7 +15466,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="s">
         <v>16</v>
       </c>
@@ -15528,7 +15528,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="241" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="s">
         <v>16</v>
       </c>
@@ -15590,7 +15590,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
         <v>17</v>
       </c>
@@ -15652,7 +15652,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="243" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
         <v>17</v>
       </c>
@@ -15714,7 +15714,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
         <v>17</v>
       </c>
@@ -15776,7 +15776,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="245" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
         <v>17</v>
       </c>
@@ -15838,7 +15838,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
         <v>17</v>
       </c>
@@ -15900,7 +15900,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="247" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="s">
         <v>17</v>
       </c>
@@ -15962,7 +15962,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
         <v>17</v>
       </c>
@@ -16024,7 +16024,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="s">
         <v>17</v>
       </c>
@@ -16086,7 +16086,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="s">
         <v>17</v>
       </c>
@@ -16148,7 +16148,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="s">
         <v>17</v>
       </c>
@@ -16210,7 +16210,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="252" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A252" s="1" t="s">
         <v>17</v>
       </c>
@@ -16272,7 +16272,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="s">
         <v>17</v>
       </c>
@@ -16334,7 +16334,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="254" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A254" s="1" t="s">
         <v>17</v>
       </c>
@@ -16396,7 +16396,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="s">
         <v>17</v>
       </c>
@@ -16458,7 +16458,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="256" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="s">
         <v>17</v>
       </c>
@@ -16520,7 +16520,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="257" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A257" s="1" t="s">
         <v>17</v>
       </c>
@@ -16582,7 +16582,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="258" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A258" s="1" t="s">
         <v>17</v>
       </c>
@@ -16644,7 +16644,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="259" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="s">
         <v>17</v>
       </c>
@@ -16706,7 +16706,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="260" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A260" s="1" t="s">
         <v>17</v>
       </c>
@@ -16768,7 +16768,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A261" s="1" t="s">
         <v>17</v>
       </c>
@@ -16830,7 +16830,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="262" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A262" s="1" t="s">
         <v>17</v>
       </c>
@@ -16892,7 +16892,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="263" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A263" s="1" t="s">
         <v>17</v>
       </c>
@@ -16954,7 +16954,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="264" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A264" s="1" t="s">
         <v>17</v>
       </c>
@@ -17016,7 +17016,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="265" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A265" s="1" t="s">
         <v>17</v>
       </c>
@@ -17078,7 +17078,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="266" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A266" s="1" t="s">
         <v>17</v>
       </c>
@@ -17140,7 +17140,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A267" s="1" t="s">
         <v>17</v>
       </c>
@@ -17202,7 +17202,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="268" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A268" s="1" t="s">
         <v>17</v>
       </c>
@@ -17264,7 +17264,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="269" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A269" s="1" t="s">
         <v>17</v>
       </c>
@@ -17326,7 +17326,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="270" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A270" s="1" t="s">
         <v>17</v>
       </c>
@@ -17388,7 +17388,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="271" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="s">
         <v>17</v>
       </c>
@@ -17450,7 +17450,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="272" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A272" s="1" t="s">
         <v>17</v>
       </c>
@@ -17512,7 +17512,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="273" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A273" s="1" t="s">
         <v>17</v>
       </c>
@@ -17574,7 +17574,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="274" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A274" s="1" t="s">
         <v>17</v>
       </c>
@@ -17636,7 +17636,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="275" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="s">
         <v>17</v>
       </c>
@@ -17698,7 +17698,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="276" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A276" s="1" t="s">
         <v>17</v>
       </c>
@@ -17760,7 +17760,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="277" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A277" s="1" t="s">
         <v>17</v>
       </c>
@@ -17822,7 +17822,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="278" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A278" s="1" t="s">
         <v>17</v>
       </c>
@@ -17884,7 +17884,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="279" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A279" s="1" t="s">
         <v>17</v>
       </c>
@@ -17946,7 +17946,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="280" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A280" s="1" t="s">
         <v>17</v>
       </c>
@@ -18008,7 +18008,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="281" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A281" s="1" t="s">
         <v>17</v>
       </c>
@@ -18070,7 +18070,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="282" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A282" s="1" t="s">
         <v>18</v>
       </c>
@@ -18132,7 +18132,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="283" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A283" s="1" t="s">
         <v>18</v>
       </c>
@@ -18194,7 +18194,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="284" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A284" s="1" t="s">
         <v>18</v>
       </c>
@@ -18256,7 +18256,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="285" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A285" s="1" t="s">
         <v>18</v>
       </c>
@@ -18318,7 +18318,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="286" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A286" s="1" t="s">
         <v>18</v>
       </c>
@@ -18380,7 +18380,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="287" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="s">
         <v>18</v>
       </c>
@@ -18442,7 +18442,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="288" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A288" s="1" t="s">
         <v>18</v>
       </c>
@@ -18504,7 +18504,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="289" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A289" s="1" t="s">
         <v>18</v>
       </c>
@@ -18566,7 +18566,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="290" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A290" s="1" t="s">
         <v>18</v>
       </c>
@@ -18628,7 +18628,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="291" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A291" s="1" t="s">
         <v>18</v>
       </c>
@@ -18690,7 +18690,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="292" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A292" s="1" t="s">
         <v>18</v>
       </c>
@@ -18752,7 +18752,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="293" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A293" s="1" t="s">
         <v>18</v>
       </c>
@@ -18814,7 +18814,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="294" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A294" s="1" t="s">
         <v>18</v>
       </c>
@@ -18876,7 +18876,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="295" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A295" s="1" t="s">
         <v>18</v>
       </c>
@@ -18938,7 +18938,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="296" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A296" s="1" t="s">
         <v>18</v>
       </c>
@@ -19000,7 +19000,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="297" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A297" s="1" t="s">
         <v>18</v>
       </c>
@@ -19062,7 +19062,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="298" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A298" s="1" t="s">
         <v>18</v>
       </c>
@@ -19124,7 +19124,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="299" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A299" s="1" t="s">
         <v>18</v>
       </c>
@@ -19186,7 +19186,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="300" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A300" s="1" t="s">
         <v>18</v>
       </c>
@@ -19248,7 +19248,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="301" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A301" s="1" t="s">
         <v>18</v>
       </c>
@@ -19310,7 +19310,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="302" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A302" s="1" t="s">
         <v>18</v>
       </c>
@@ -19372,7 +19372,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="303" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A303" s="1" t="s">
         <v>18</v>
       </c>
@@ -19434,7 +19434,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="304" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A304" s="1" t="s">
         <v>18</v>
       </c>
@@ -19496,7 +19496,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="305" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A305" s="1" t="s">
         <v>18</v>
       </c>
@@ -19558,7 +19558,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="306" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A306" s="1" t="s">
         <v>18</v>
       </c>
@@ -19620,7 +19620,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="307" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A307" s="1" t="s">
         <v>18</v>
       </c>
@@ -19682,7 +19682,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="308" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A308" s="1" t="s">
         <v>18</v>
       </c>
@@ -19744,7 +19744,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="309" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A309" s="1" t="s">
         <v>18</v>
       </c>
@@ -19806,7 +19806,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="310" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A310" s="1" t="s">
         <v>18</v>
       </c>
@@ -19868,7 +19868,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="311" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A311" s="1" t="s">
         <v>18</v>
       </c>
@@ -19930,7 +19930,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="312" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A312" s="1" t="s">
         <v>18</v>
       </c>
@@ -19992,7 +19992,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="313" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A313" s="1" t="s">
         <v>18</v>
       </c>
@@ -20054,7 +20054,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="314" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A314" s="1" t="s">
         <v>18</v>
       </c>
@@ -20116,7 +20116,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="315" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A315" s="1" t="s">
         <v>18</v>
       </c>
@@ -20178,7 +20178,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="316" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A316" s="1" t="s">
         <v>18</v>
       </c>
@@ -20240,7 +20240,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="317" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A317" s="1" t="s">
         <v>18</v>
       </c>
@@ -20302,7 +20302,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="318" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A318" s="1" t="s">
         <v>18</v>
       </c>
@@ -20364,7 +20364,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="319" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A319" s="1" t="s">
         <v>18</v>
       </c>
@@ -20426,7 +20426,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="320" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A320" s="1" t="s">
         <v>18</v>
       </c>
@@ -20488,7 +20488,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="321" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A321" s="1" t="s">
         <v>18</v>
       </c>
@@ -20550,7 +20550,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="322" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A322" s="1" t="s">
         <v>19</v>
       </c>
@@ -20612,7 +20612,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="323" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A323" s="1" t="s">
         <v>19</v>
       </c>
@@ -20674,7 +20674,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="324" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A324" s="1" t="s">
         <v>19</v>
       </c>
@@ -20736,7 +20736,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="325" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A325" s="1" t="s">
         <v>19</v>
       </c>
@@ -20798,7 +20798,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="326" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A326" s="1" t="s">
         <v>19</v>
       </c>
@@ -20860,7 +20860,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="327" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A327" s="1" t="s">
         <v>19</v>
       </c>
@@ -20922,7 +20922,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="328" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A328" s="1" t="s">
         <v>19</v>
       </c>
@@ -20984,7 +20984,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="329" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A329" s="1" t="s">
         <v>19</v>
       </c>
@@ -21046,7 +21046,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="330" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A330" s="1" t="s">
         <v>19</v>
       </c>
@@ -21108,7 +21108,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="331" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A331" s="1" t="s">
         <v>19</v>
       </c>
@@ -21170,7 +21170,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="332" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A332" s="1" t="s">
         <v>19</v>
       </c>
@@ -21232,7 +21232,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="333" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A333" s="1" t="s">
         <v>19</v>
       </c>
@@ -21294,7 +21294,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="334" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A334" s="1" t="s">
         <v>19</v>
       </c>
@@ -21356,7 +21356,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="335" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A335" s="1" t="s">
         <v>19</v>
       </c>
@@ -21418,7 +21418,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="336" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A336" s="1" t="s">
         <v>19</v>
       </c>
@@ -21480,7 +21480,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="337" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A337" s="1" t="s">
         <v>19</v>
       </c>
@@ -21542,7 +21542,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="338" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A338" s="1" t="s">
         <v>19</v>
       </c>
@@ -21604,7 +21604,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="339" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A339" s="1" t="s">
         <v>19</v>
       </c>
@@ -21666,7 +21666,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="340" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A340" s="1" t="s">
         <v>19</v>
       </c>
@@ -21728,7 +21728,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="341" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A341" s="1" t="s">
         <v>19</v>
       </c>
@@ -21790,7 +21790,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="342" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A342" s="1" t="s">
         <v>19</v>
       </c>
@@ -21852,7 +21852,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="343" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A343" s="1" t="s">
         <v>19</v>
       </c>
@@ -21914,7 +21914,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="344" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A344" s="1" t="s">
         <v>19</v>
       </c>
@@ -21976,7 +21976,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="345" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A345" s="1" t="s">
         <v>19</v>
       </c>
@@ -22038,7 +22038,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="346" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A346" s="1" t="s">
         <v>19</v>
       </c>
@@ -22100,7 +22100,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="347" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A347" s="1" t="s">
         <v>19</v>
       </c>
@@ -22162,7 +22162,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="348" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A348" s="1" t="s">
         <v>19</v>
       </c>
@@ -22224,7 +22224,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="349" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A349" s="1" t="s">
         <v>19</v>
       </c>
@@ -22286,7 +22286,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="350" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A350" s="1" t="s">
         <v>19</v>
       </c>
@@ -22348,7 +22348,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="351" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A351" s="1" t="s">
         <v>19</v>
       </c>
@@ -22410,7 +22410,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="352" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A352" s="1" t="s">
         <v>19</v>
       </c>
@@ -22472,7 +22472,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="353" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A353" s="1" t="s">
         <v>19</v>
       </c>
@@ -22534,7 +22534,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="354" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A354" s="1" t="s">
         <v>19</v>
       </c>
@@ -22596,7 +22596,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="355" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A355" s="1" t="s">
         <v>19</v>
       </c>
@@ -22658,7 +22658,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="356" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A356" s="1" t="s">
         <v>19</v>
       </c>
@@ -22720,7 +22720,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="357" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A357" s="1" t="s">
         <v>19</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="358" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A358" s="1" t="s">
         <v>19</v>
       </c>
@@ -22844,7 +22844,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="359" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A359" s="1" t="s">
         <v>19</v>
       </c>
@@ -22906,7 +22906,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="360" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A360" s="1" t="s">
         <v>19</v>
       </c>
@@ -22968,7 +22968,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="361" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A361" s="1" t="s">
         <v>19</v>
       </c>
@@ -23030,7 +23030,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="362" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A362" s="1" t="s">
         <v>20</v>
       </c>
@@ -23092,7 +23092,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="363" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A363" s="1" t="s">
         <v>20</v>
       </c>
@@ -23154,7 +23154,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="364" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A364" s="1" t="s">
         <v>20</v>
       </c>
@@ -23216,7 +23216,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="365" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A365" s="1" t="s">
         <v>20</v>
       </c>
@@ -23278,7 +23278,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="366" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A366" s="1" t="s">
         <v>20</v>
       </c>
@@ -23340,7 +23340,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="367" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A367" s="1" t="s">
         <v>20</v>
       </c>
@@ -23402,7 +23402,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="368" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A368" s="1" t="s">
         <v>20</v>
       </c>
@@ -23464,7 +23464,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="369" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A369" s="1" t="s">
         <v>20</v>
       </c>
@@ -23526,7 +23526,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="370" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A370" s="1" t="s">
         <v>20</v>
       </c>
@@ -23588,7 +23588,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="371" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A371" s="1" t="s">
         <v>20</v>
       </c>
@@ -23650,7 +23650,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="372" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A372" s="1" t="s">
         <v>20</v>
       </c>
@@ -23712,7 +23712,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="373" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A373" s="1" t="s">
         <v>20</v>
       </c>
@@ -23774,7 +23774,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="374" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A374" s="1" t="s">
         <v>20</v>
       </c>
@@ -23836,7 +23836,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="375" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A375" s="1" t="s">
         <v>20</v>
       </c>
@@ -23898,7 +23898,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="376" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A376" s="1" t="s">
         <v>20</v>
       </c>
@@ -23960,7 +23960,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="377" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A377" s="1" t="s">
         <v>20</v>
       </c>
@@ -24022,7 +24022,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="378" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A378" s="1" t="s">
         <v>20</v>
       </c>
@@ -24084,7 +24084,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="379" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A379" s="1" t="s">
         <v>20</v>
       </c>
@@ -24146,7 +24146,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="380" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A380" s="1" t="s">
         <v>20</v>
       </c>
@@ -24208,7 +24208,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="381" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A381" s="1" t="s">
         <v>20</v>
       </c>
@@ -24270,7 +24270,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="382" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A382" s="1" t="s">
         <v>20</v>
       </c>
@@ -24332,7 +24332,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="383" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A383" s="1" t="s">
         <v>20</v>
       </c>
@@ -24394,7 +24394,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="384" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A384" s="1" t="s">
         <v>20</v>
       </c>
@@ -24456,7 +24456,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="385" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A385" s="1" t="s">
         <v>20</v>
       </c>
@@ -24518,7 +24518,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="386" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A386" s="1" t="s">
         <v>20</v>
       </c>
@@ -24580,7 +24580,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="387" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A387" s="1" t="s">
         <v>20</v>
       </c>
@@ -24642,7 +24642,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="388" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A388" s="1" t="s">
         <v>20</v>
       </c>
@@ -24704,7 +24704,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="389" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A389" s="1" t="s">
         <v>20</v>
       </c>
@@ -24766,7 +24766,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="390" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A390" s="1" t="s">
         <v>20</v>
       </c>
@@ -24828,7 +24828,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="391" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A391" s="1" t="s">
         <v>20</v>
       </c>
@@ -24890,7 +24890,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="392" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A392" s="1" t="s">
         <v>20</v>
       </c>
@@ -24952,7 +24952,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="393" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A393" s="1" t="s">
         <v>20</v>
       </c>
@@ -25014,7 +25014,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="394" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A394" s="1" t="s">
         <v>20</v>
       </c>
@@ -25076,7 +25076,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="395" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A395" s="1" t="s">
         <v>20</v>
       </c>
@@ -25138,7 +25138,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="396" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A396" s="1" t="s">
         <v>20</v>
       </c>
@@ -25200,7 +25200,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="397" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A397" s="1" t="s">
         <v>20</v>
       </c>
@@ -25262,7 +25262,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="398" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A398" s="1" t="s">
         <v>20</v>
       </c>
@@ -25324,7 +25324,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="399" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A399" s="1" t="s">
         <v>20</v>
       </c>
@@ -25386,7 +25386,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="400" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A400" s="1" t="s">
         <v>20</v>
       </c>
@@ -25448,7 +25448,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="401" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A401" s="1" t="s">
         <v>20</v>
       </c>
@@ -25517,6 +25517,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="92bd62ed-fc4d-4ee3-b38b-98b6ea89ea27">
@@ -25537,15 +25546,6 @@
     </SharedWithUsers>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25772,20 +25772,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57442DEA-E7F2-4A83-BE05-0FDE7066AD8E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F81A3C2A-7321-4847-85BE-BA2A09CFC8B6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="92bd62ed-fc4d-4ee3-b38b-98b6ea89ea27"/>
     <ds:schemaRef ds:uri="87753393-e6c0-4d5a-be47-99eb96ae390c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57442DEA-E7F2-4A83-BE05-0FDE7066AD8E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>